<commit_message>
feat: implement JWT token authentication and migrate users
</commit_message>
<xml_diff>
--- a/fast_api/vaxflow_synthesized_dataset_final.xlsx
+++ b/fast_api/vaxflow_synthesized_dataset_final.xlsx
@@ -19794,13 +19794,13 @@
         <v>5</v>
       </c>
       <c r="C198" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D198" t="n">
         <v>140</v>
       </c>
       <c r="E198" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F198" t="n">
         <v>34.1</v>
@@ -19818,25 +19818,25 @@
         <v>0.6899999999999999</v>
       </c>
       <c r="K198" t="n">
-        <v>563</v>
+        <v>500</v>
       </c>
       <c r="L198" t="n">
-        <v>56</v>
+        <v>300</v>
       </c>
       <c r="M198" t="n">
-        <v>122</v>
+        <v>100</v>
       </c>
       <c r="N198" t="n">
-        <v>12</v>
+        <v>100</v>
       </c>
       <c r="O198" t="n">
-        <v>1256</v>
+        <v>2999</v>
       </c>
       <c r="P198" t="n">
         <v>117</v>
       </c>
       <c r="Q198" t="n">
-        <v>0.89</v>
+        <v>0.79</v>
       </c>
       <c r="R198" t="n">
         <v>0</v>
@@ -19851,13 +19851,13 @@
         <v>0</v>
       </c>
       <c r="V198" t="n">
-        <v>0.91</v>
+        <v>0.95</v>
       </c>
       <c r="W198" t="n">
         <v>0.89</v>
       </c>
       <c r="X198" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Y198" t="n">
         <v>0</v>
@@ -19875,7 +19875,7 @@
         <v>6.9</v>
       </c>
       <c r="AD198" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE198" t="n">
         <v>0</v>

</xml_diff>